<commit_message>
Configuracion WAN (Ruteo entre TGU - SPS / SPS - TGU)
</commit_message>
<xml_diff>
--- a/DIRECCIONAMIENTO WAN.xlsx
+++ b/DIRECCIONAMIENTO WAN.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Leonel\Proyecto Redes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{308701E6-B4F3-4689-8254-6AA15D03F7DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{345842FB-535F-4ECE-95D5-792DE0B1FFE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{3FF35EE7-BEA4-4846-9613-473D9BEE8700}"/>
+    <workbookView xWindow="3250" yWindow="1600" windowWidth="14400" windowHeight="7270" activeTab="1" xr2:uid="{3FF35EE7-BEA4-4846-9613-473D9BEE8700}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="RUTEOS" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="82">
   <si>
     <t>DIRECCIONAMIENTO REDES WAN</t>
   </si>
@@ -183,6 +184,108 @@
   </si>
   <si>
     <t>10.10.0.31</t>
+  </si>
+  <si>
+    <t>TABLA RUTEO PAN - CR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SALTO </t>
+  </si>
+  <si>
+    <t>184.168.5.0</t>
+  </si>
+  <si>
+    <t>184.168.5.32</t>
+  </si>
+  <si>
+    <t>184.168.5.64</t>
+  </si>
+  <si>
+    <t>TABLA RUTEO CR - PAN</t>
+  </si>
+  <si>
+    <t>SALTO</t>
+  </si>
+  <si>
+    <t>255.255.255.224</t>
+  </si>
+  <si>
+    <t>255.255.255.248</t>
+  </si>
+  <si>
+    <t>185.168.6.0</t>
+  </si>
+  <si>
+    <t>185.168.6.32</t>
+  </si>
+  <si>
+    <t>185.168.6.64</t>
+  </si>
+  <si>
+    <t>RED DESTINO</t>
+  </si>
+  <si>
+    <t>TABLA RUTEO NYK - ATL</t>
+  </si>
+  <si>
+    <t>TABLA RUTEO ATL - NYK</t>
+  </si>
+  <si>
+    <t>9.9.9.0</t>
+  </si>
+  <si>
+    <t>255.255.255.128</t>
+  </si>
+  <si>
+    <t>9.9.9.128</t>
+  </si>
+  <si>
+    <t>255.255.255.192</t>
+  </si>
+  <si>
+    <t>9.9.10.0</t>
+  </si>
+  <si>
+    <t>9.9.9.192</t>
+  </si>
+  <si>
+    <t>9.9.10.8</t>
+  </si>
+  <si>
+    <t>8.8.8.0</t>
+  </si>
+  <si>
+    <t>8.8.8.8</t>
+  </si>
+  <si>
+    <t>TABLA RUTEO TGU -SPS</t>
+  </si>
+  <si>
+    <t>TABLA RUTEO SPS - TGU</t>
+  </si>
+  <si>
+    <t>181.168.2.0</t>
+  </si>
+  <si>
+    <t>181.168.2.64</t>
+  </si>
+  <si>
+    <t>181.168.2.112</t>
+  </si>
+  <si>
+    <t>181.168.2.96</t>
+  </si>
+  <si>
+    <t>255.255.255.240</t>
+  </si>
+  <si>
+    <t>180.168.1.0</t>
+  </si>
+  <si>
+    <t>180.168.1.128</t>
+  </si>
+  <si>
+    <t>180.168.1.192</t>
   </si>
 </sst>
 </file>
@@ -759,4 +862,308 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F54AF1A9-5D53-410E-B4FB-3B69DB7B9DAA}">
+  <dimension ref="A1:O15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.81640625" customWidth="1"/>
+    <col min="5" max="5" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.26953125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.7265625" customWidth="1"/>
+    <col min="13" max="13" width="20" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I1" t="s">
+        <v>62</v>
+      </c>
+      <c r="M1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J2" t="s">
+        <v>60</v>
+      </c>
+      <c r="K2" t="s">
+        <v>5</v>
+      </c>
+      <c r="M2" t="s">
+        <v>54</v>
+      </c>
+      <c r="N2" t="s">
+        <v>60</v>
+      </c>
+      <c r="O2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" t="s">
+        <v>55</v>
+      </c>
+      <c r="I3" t="s">
+        <v>44</v>
+      </c>
+      <c r="J3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K3" t="s">
+        <v>64</v>
+      </c>
+      <c r="M3" t="s">
+        <v>41</v>
+      </c>
+      <c r="N3" t="s">
+        <v>70</v>
+      </c>
+      <c r="O3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>58</v>
+      </c>
+      <c r="G4" t="s">
+        <v>55</v>
+      </c>
+      <c r="I4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J4" t="s">
+        <v>65</v>
+      </c>
+      <c r="K4" t="s">
+        <v>66</v>
+      </c>
+      <c r="M4" t="s">
+        <v>41</v>
+      </c>
+      <c r="N4" t="s">
+        <v>71</v>
+      </c>
+      <c r="O4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" t="s">
+        <v>56</v>
+      </c>
+      <c r="I5" t="s">
+        <v>44</v>
+      </c>
+      <c r="J5" t="s">
+        <v>67</v>
+      </c>
+      <c r="K5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="I6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J6" t="s">
+        <v>68</v>
+      </c>
+      <c r="K6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="I7" t="s">
+        <v>44</v>
+      </c>
+      <c r="J7" t="s">
+        <v>69</v>
+      </c>
+      <c r="K7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>72</v>
+      </c>
+      <c r="E10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" t="s">
+        <v>5</v>
+      </c>
+      <c r="E11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>79</v>
+      </c>
+      <c r="G12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" t="s">
+        <v>81</v>
+      </c>
+      <c r="G14" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15" t="s">
+        <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>